<commit_message>
refactor: first as independent stage + media preview (v1.11.0)
</commit_message>
<xml_diff>
--- a/EDGE7/templates/EDGE-Pack/EDGE-内容.xlsx
+++ b/EDGE7/templates/EDGE-Pack/EDGE-内容.xlsx
@@ -21,18 +21,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00CC0000"/>
-      <sz val="14"/>
     </font>
     <font>
       <b val="1"/>
@@ -52,7 +47,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -60,33 +55,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00CCCCCC"/>
-      </left>
-      <right style="thin">
-        <color rgb="00CCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00CCCCCC"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -452,88 +427,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="88" customWidth="1" min="1" max="1"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>EDGE-Infinity 内容模板（单次游玩可上传本文件）</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>用法：</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>1. 按四个阶段工作表填写：开场 / go / stop / finish</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2. 在网页选项页选择本 xlsx →「加载表格（仅本局）」；数据只在浏览器内存，不会上传到服务器</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>3. 不加载则使用网站默认内容</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>4. 语音仍使用网站 audio/{阶段}/{阶段}_{编号}.wav（编号列 = audioIdx，从 0 起）</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>5. 图片可选：填写相对路径如 images/go/01.webp（需文件已在站点或后续资料包中）</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>finish 颜色：green = 允许释放；red = 不允许释放</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>标签 tags：多个用英文逗号分隔，如 edge,prostate</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>请勿改工作表名称。留空行会被忽略。</t>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>first 为独立阶段，语音用 first_N.wav，不要再用 go_N 代替开场</t>
         </is>
       </c>
     </row>
@@ -548,54 +448,51 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>编号audioIdx</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>文案</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>秒数</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>fps</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>图片路径</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>视频路径</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="80" customHeight="1">
+    <row r="2">
       <c r="A2" t="n">
         <v>0</v>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>&lt;small&gt;任务开始！&lt;br /&gt;贱狗，现在可以开始慢慢撸你的狗鸡巴了。&lt;br /&gt;游戏过程中会随机出现各种羞辱指令。&lt;br /&gt;当进度条进入边缘区时，你要拼命接近高潮或潮吹的极限，但绝对不准射出来！&lt;br /&gt;记住：你这根贱狗鸡巴永远没有自行排精的权利，一切都由主人决定。&lt;/small&gt;</t>
         </is>
@@ -609,7 +506,12 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>开场语音实际播放 go_{编号}.wav</t>
+          <t>video/first/first_0.mp4</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>独立 first</t>
         </is>
       </c>
     </row>
@@ -626,58 +528,49 @@
   </sheetPr>
   <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="56" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>编号audioIdx</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>文案</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>秒数</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>fps</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>标签tags</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>图片路径</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="36" customHeight="1">
+    <row r="2">
       <c r="A2" t="n">
         <v>0</v>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>现在开始慢慢撸你的贱狗鸡巴，让它给我彻底硬起来，好好感受主人对你的绝对控制</t>
         </is>
@@ -696,11 +589,11 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
     </row>
-    <row r="3" ht="36" customHeight="1">
+    <row r="3">
       <c r="A3" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>用最快的速度疯狂撸管！像条发情的母狗一样，给老子用力点！</t>
         </is>
@@ -719,11 +612,11 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
     </row>
-    <row r="4" ht="36" customHeight="1">
+    <row r="4">
       <c r="A4" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>加速！把你的狗屌撸到又烫又红，卖力点，别偷懒！</t>
         </is>
@@ -742,11 +635,11 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
     </row>
-    <row r="5" ht="36" customHeight="1">
+    <row r="5">
       <c r="A5" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>贱狗是不是已经很想射了？继续撸，别停！把那股射意给老子狠狠憋住！</t>
         </is>
@@ -765,11 +658,11 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
     </row>
-    <row r="6" ht="36" customHeight="1">
+    <row r="6">
       <c r="A6" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>快到极限了吧？死死给我憋住！再快一点，你这没用的贱货！</t>
         </is>
@@ -788,11 +681,11 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
     </row>
-    <row r="7" ht="36" customHeight="1">
+    <row r="7">
       <c r="A7" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>一只手疯狂撸鸡巴，另一只手用力捏你的狗蛋！疼也要继续撸下去！</t>
         </is>
@@ -811,11 +704,11 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
     </row>
-    <row r="8" ht="36" customHeight="1">
+    <row r="8">
       <c r="A8" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>大声叫出来：“主人，贱狗好想射！请主人可怜可怜我！”边叫边撸</t>
         </is>
@@ -834,11 +727,11 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
     </row>
-    <row r="9" ht="36" customHeight="1">
+    <row r="9">
       <c r="A9" t="n">
         <v>7</v>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>扇自己十个响亮的耳光，同时继续疯狂撸管，不准停手！</t>
         </is>
@@ -857,11 +750,11 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
     </row>
-    <row r="10" ht="36" customHeight="1">
+    <row r="10">
       <c r="A10" t="n">
         <v>8</v>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>现在全力加速冲刺！你的狗鸡巴是不是快要喷了？给老子死死憋住！</t>
         </is>
@@ -880,11 +773,11 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
     </row>
-    <row r="11" ht="36" customHeight="1">
+    <row r="11">
       <c r="A11" t="n">
         <v>9</v>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>用力捏紧你的两个乳头狠狠拧转！边疼边撸，越疼越兴奋！</t>
         </is>
@@ -903,11 +796,11 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
     </row>
-    <row r="12" ht="36" customHeight="1">
+    <row r="12">
       <c r="A12" t="n">
         <v>10</v>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>双手抱头，只用腰部疯狂挺动狗鸡巴，像条发情的母狗在操空气一样下贱！</t>
         </is>
@@ -926,11 +819,11 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
     </row>
-    <row r="13" ht="36" customHeight="1">
+    <row r="13">
       <c r="A13" t="n">
         <v>11</v>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>只用指尖快速上下摩擦龟头下面的系带，绕圈或者轻轻刮，拼命接近高潮，但绝对不准射出来！好好感受那股直冲脑门的耻辱快感</t>
         </is>
@@ -949,11 +842,11 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
     </row>
-    <row r="14" ht="36" customHeight="1">
+    <row r="14">
       <c r="A14" t="n">
         <v>12</v>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>用拇指轻轻刮弄马眼口，同时快速撸管，体会你这贱狗的尿道被玩弄的羞耻感觉，边缘到极限再慢下来</t>
         </is>
@@ -972,11 +865,11 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
     </row>
-    <row r="15" ht="36" customHeight="1">
+    <row r="15">
       <c r="A15" t="n">
         <v>13</v>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>集中攻击你的龟背！用两根手指用力轻刮或按压那根敏感的系带，边刺激边大声说“龟背是主人的”</t>
         </is>
@@ -995,11 +888,11 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr"/>
     </row>
-    <row r="16" ht="36" customHeight="1">
+    <row r="16">
       <c r="A16" t="n">
         <v>14</v>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>贱狗，把一根手指涂满口水，慢慢插进你的骚屁眼，用“来这里”的勾指动作按摩前列腺，边勾边撸鸡巴，给我好好挑战潮吹边缘</t>
         </is>
@@ -1018,11 +911,11 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
     </row>
-    <row r="17" ht="36" customHeight="1">
+    <row r="17">
       <c r="A17" t="n">
         <v>15</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>用中指在屁眼里画圈或轻敲前列腺，同时快速撸管，感受前列腺液马上要喷出来的强烈尿意，但绝对不准给老子释放！</t>
         </is>
@@ -1041,11 +934,11 @@
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
     </row>
-    <row r="18" ht="36" customHeight="1">
+    <row r="18">
       <c r="A18" t="n">
         <v>16</v>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>跪好，一根手指插进骚屁眼，反复抽插并用力勾前列腺，像主人正在榨你的前列腺奶一样，边玩边喊“贱狗的屁眼是主人的玩具”</t>
         </is>
@@ -1064,11 +957,11 @@
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr"/>
     </row>
-    <row r="19" ht="36" customHeight="1">
+    <row r="19">
       <c r="A19" t="n">
         <v>17</v>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>用手指用力反复按压会阴，刺激你里面的前列腺，体会你这贱狗被外部遥控的耻辱感觉</t>
         </is>
@@ -1087,11 +980,11 @@
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
     </row>
-    <row r="20" ht="36" customHeight="1">
+    <row r="20">
       <c r="A20" t="n">
         <v>18</v>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>双重刺激！一只手专攻龟背和马眼，另一只手指插进屁眼勾前列腺，拼命边缘，却不准喷出任何液体！</t>
         </is>
@@ -1110,11 +1003,11 @@
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
     </row>
-    <row r="21" ht="36" customHeight="1">
+    <row r="21">
       <c r="A21" t="n">
         <v>19</v>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>把鸡巴整根插进飞机杯里疯狂抽插，同时手指玩弄你的骚屁眼按摩前列腺，体验前后都被操的强烈耻辱感</t>
         </is>
@@ -1133,11 +1026,11 @@
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
     </row>
-    <row r="22" ht="36" customHeight="1">
+    <row r="22">
       <c r="A22" t="n">
         <v>20</v>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>潮吹边缘加强！手指在屁眼里用力勾前列腺，另一只手刮龟背和马眼，接近要喷前列腺液的极限，却给老子死死憋住！</t>
         </is>
@@ -1169,52 +1062,44 @@
   </sheetPr>
   <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="56" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>编号audioIdx</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>文案</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>秒数</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>标签tags</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>图片路径</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="36" customHeight="1">
+    <row r="2">
       <c r="A2" t="n">
         <v>0</v>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>立刻把手从你的贱狗鸡巴上拿开！不准再碰一下！</t>
         </is>
@@ -1230,11 +1115,11 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
     </row>
-    <row r="3" ht="36" customHeight="1">
+    <row r="3">
       <c r="A3" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>停止一切动作！双手抱头，深呼吸，狠狠憋住那股想射的冲动！</t>
         </is>
@@ -1250,11 +1135,11 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
     </row>
-    <row r="4" ht="36" customHeight="1">
+    <row r="4">
       <c r="A4" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>立刻扇自己十个响亮耳光！一边扇一边大声说“贱狗不配射精”</t>
         </is>
@@ -1270,11 +1155,11 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
     </row>
-    <row r="5" ht="36" customHeight="1">
+    <row r="5">
       <c r="A5" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>停止撸管！大声喊二十遍“主人，贱狗听话，不敢射！”</t>
         </is>
@@ -1290,11 +1175,11 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
     </row>
-    <row r="6" ht="36" customHeight="1">
+    <row r="6">
       <c r="A6" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>把手拿开，让你的狗鸡巴在空气中可怜地一跳一跳地求饶</t>
         </is>
@@ -1310,11 +1195,11 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
     </row>
-    <row r="7" ht="36" customHeight="1">
+    <row r="7">
       <c r="A7" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>贱狗无权排精！立刻停止，跪直身体好好反省自己的下贱</t>
         </is>
@@ -1330,11 +1215,11 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
     </row>
-    <row r="8" ht="36" customHeight="1">
+    <row r="8">
       <c r="A8" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>现在用力拧自己的乳头，同时说“谢谢主人不让我射”</t>
         </is>
@@ -1350,11 +1235,11 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
     </row>
-    <row r="9" ht="36" customHeight="1">
+    <row r="9">
       <c r="A9" t="n">
         <v>7</v>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>停止所有动作！把插在骚屁眼里的手指慢慢拔出来，感受前列腺被玩弄后那空虚又跳动的耻辱</t>
         </is>
@@ -1370,11 +1255,11 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
     </row>
-    <row r="10" ht="36" customHeight="1">
+    <row r="10">
       <c r="A10" t="n">
         <v>8</v>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>把手拿开！继续用手指轻轻按压会阴，体会前列腺还在疯狂求饶却不准释放的痛苦</t>
         </is>
@@ -1390,11 +1275,11 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
     </row>
-    <row r="11" ht="36" customHeight="1">
+    <row r="11">
       <c r="A11" t="n">
         <v>9</v>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>立刻停止龟背和屁眼的所有刺激！跪好反省：“贱狗的龟背、马眼和骚屁眼都不配高潮”</t>
         </is>
@@ -1410,11 +1295,11 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
     </row>
-    <row r="12" ht="36" customHeight="1">
+    <row r="12">
       <c r="A12" t="n">
         <v>10</v>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>停！手指从屁眼里拔出来后，高高翘起屁股，让你的骚屁眼一张一合，展示被玩弄过的下贱模样</t>
         </is>
@@ -1443,64 +1328,54 @@
   </sheetPr>
   <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="52" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>编号audioIdx</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>文案</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>秒数</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>颜色green或red</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>fps</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>标签tags</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>图片路径</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="40" customHeight="1">
+    <row r="2">
       <c r="A2" t="n">
         <v>0</v>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>停！这次主人心情不好，贱狗不准排精。&lt;br /&gt;把手从狗屌上拿开，让它慢慢软下去吧，你这可怜又没用的废物！</t>
         </is>
@@ -1521,18 +1396,12 @@
           <t>deny</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>green=允许 red=不允许</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="40" customHeight="1">
+    </row>
+    <row r="3">
       <c r="A3" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>射！现在立刻给老子射出来！把所有精液都喷得干干净净！</t>
         </is>
@@ -1553,18 +1422,12 @@
           <t>allow</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>green=允许 red=不允许</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="40" customHeight="1">
+    </row>
+    <row r="4">
       <c r="A4" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>慢慢射……每一滴都要射得又慢又彻底</t>
         </is>
@@ -1585,18 +1448,12 @@
           <t>allow</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>green=允许 red=不允许</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="40" customHeight="1">
+    </row>
+    <row r="5">
       <c r="A5" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>射！用你最淫荡、最下贱的方式射精！边射边大声喊主人的名字！</t>
         </is>
@@ -1617,18 +1474,12 @@
           <t>allow</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>green=允许 red=不允许</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="40" customHeight="1">
+    </row>
+    <row r="6">
       <c r="A6" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>给我射！贱狗只有8秒钟时间，否则就永远给我憋着！快点！</t>
         </is>
@@ -1649,18 +1500,12 @@
           <t>allow</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>green=允许 red=不允许</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="40" customHeight="1">
+    </row>
+    <row r="7">
       <c r="A7" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>贱狗可以射了！快点把精液全部奉献给主人，射得越狼狈越好！</t>
         </is>
@@ -1681,18 +1526,12 @@
           <t>allow</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>green=允许 red=不允许</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="40" customHeight="1">
+    </row>
+    <row r="8">
       <c r="A8" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>射！射完后立刻感谢主人：“谢谢主人恩准贱狗排精”</t>
         </is>
@@ -1713,18 +1552,12 @@
           <t>allow</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>green=允许 red=不允许</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="40" customHeight="1">
+    </row>
+    <row r="9">
       <c r="A9" t="n">
         <v>7</v>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>射！把所有精液喷在自己身上，展示你这贱狗的下贱模样</t>
         </is>
@@ -1745,18 +1578,12 @@
           <t>allow</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>green=允许 red=不允许</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="40" customHeight="1">
+    </row>
+    <row r="10">
       <c r="A10" t="n">
         <v>8</v>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>射！给我潮吹出来！边射边用手指勾屁眼里的前列腺，把前列腺液和精液一起给我喷出来！</t>
         </is>
@@ -1775,12 +1602,6 @@
       <c r="F10" t="inlineStr">
         <is>
           <t>allow,prostate</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>green=允许 red=不允许</t>
         </is>
       </c>
     </row>

</xml_diff>